<commit_message>
Node changes made during completion of initial release test file completion
</commit_message>
<xml_diff>
--- a/Autogen/TestMemoryMap.xlsx
+++ b/Autogen/TestMemoryMap.xlsx
@@ -5,11 +5,12 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Test1" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Test2" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Test3" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="114">
   <si>
     <t xml:space="preserve">Member ID</t>
   </si>
@@ -147,6 +148,222 @@
   </si>
   <si>
     <t xml:space="preserve">WRITE FLOAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT8 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT8 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT8 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT8 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT8 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT8 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT8 7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT8 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT8 9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT8 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT8 11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT8 12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT8 13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT8 14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT8 15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT8 16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT8 17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT8 18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT8 19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT8 20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT32 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT32 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT32 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT32 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT32 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT32 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT32 7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT32 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT32 9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT32 10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT32 11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT32 12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT32 13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT32 14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT32 15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT32 16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT32 17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT32 18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT32 19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WRITE UINT32 20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">39</t>
   </si>
 </sst>
 </file>
@@ -1328,4 +1545,1118 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:I41"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15.81"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="18.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="13.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="27.49"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I3" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I4" s="3"/>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I5" s="3"/>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="H24" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="H25" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="H27" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G28" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="H28" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="H29" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G30" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="H30" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G31" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="H31" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G32" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="H32" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G33" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="H33" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="H34" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="H35" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G36" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G37" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="H37" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G38" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G39" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="H39" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G40" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G41" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="H41" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C2:C41" type="list">
+      <formula1>"RO,RW"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B2:B41" type="list">
+      <formula1>"uint8_t,int8_t,uint16_t,int16_t,uint32_t,int32_t,float"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H2:H41" type="list">
+      <formula1>"true,false"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>